<commit_message>
Fix WLS ATS frame orientation and lookup mappings
</commit_message>
<xml_diff>
--- a/wls_program/src/WildlifeSweeps/wildlife_parsing_codex_lookup.xlsx
+++ b/wls_program/src/WildlifeSweeps/wildlife_parsing_codex_lookup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpeciesFindingTypes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecognitionKeywords" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecognitionRegex" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skips" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SpeciesFindingTypes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RecognitionKeywords" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RecognitionRegex" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Skips" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B88"/>
+  <dimension ref="A1:B91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1484,6 +1484,42 @@
       <c r="B88" t="inlineStr">
         <is>
           <t>Sighting</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Squirrel</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Burrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Feeding</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8475,6 +8511,56 @@
       <c r="E279" t="inlineStr">
         <is>
           <t>Trail (Unidentified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>10</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>hare burrow</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Burrow</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare burrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>10</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>rabbit feeding</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Feeding</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Feeding</t>
         </is>
       </c>
     </row>
@@ -8489,7 +8575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8608,7 +8694,6 @@
           <t>Moose Hair / Fur</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8634,7 +8719,6 @@
           <t>Abandoned / Inactive Bird Nest</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8660,7 +8744,6 @@
           <t>Buck Brushing</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8686,7 +8769,6 @@
           <t>Buck Rubbing</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8712,7 +8794,6 @@
           <t>Ungulate Scrape</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8738,7 +8819,6 @@
           <t>Deer Bedding Site</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8764,7 +8844,6 @@
           <t>Deer Scat</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8790,7 +8869,6 @@
           <t>Deer Tracks</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8816,7 +8894,6 @@
           <t>Deer Trail</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -8842,7 +8919,6 @@
           <t>Rabbit Scat / Droppings</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -8868,7 +8944,6 @@
           <t>Rabbit Tracks</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -8894,7 +8969,6 @@
           <t>Rabbit Trail</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -8920,7 +8994,6 @@
           <t>Coyote Scat</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -8946,7 +9019,6 @@
           <t>Coyote Tracks</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -8972,7 +9044,6 @@
           <t>Grouse Bed</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -8998,7 +9069,6 @@
           <t>Moose Bedding Site</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9054,7 +9124,6 @@
           <t>Moose Scat</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -9080,7 +9149,6 @@
           <t>Moose Tracks</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -9106,7 +9174,6 @@
           <t>Moose Trail</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -9132,7 +9199,6 @@
           <t>Possible Bear Tracks</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -9158,7 +9224,6 @@
           <t>Woodpecker Cavity Tree</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -9184,7 +9249,6 @@
           <t>Woodpecker Feeding / Foraging Sign</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -9210,7 +9274,6 @@
           <t>Woodpecker Heard (Audible)</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -9236,7 +9299,6 @@
           <t>Woodpecker Sighting</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -9262,7 +9324,6 @@
           <t>Bedding Site (Unidentified)</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -9288,7 +9349,6 @@
           <t>Animal Remains (Species Unconfirmed)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -9314,7 +9374,6 @@
           <t>Canid Scat (Coyote/Dog)</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -9340,7 +9399,6 @@
           <t>Canid Tracks (Coyote/Dog)</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -9366,7 +9424,6 @@
           <t>Inactive / Possible Den</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -9422,7 +9479,6 @@
           <t>Ungulate Rub</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -9478,7 +9534,6 @@
           <t>Bear Scat</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -9504,7 +9559,6 @@
           <t>Possible Bear Tracks</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -9530,7 +9584,6 @@
           <t>Beaver Chew</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -9616,7 +9669,6 @@
           <t>Dog Tracks</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -9642,7 +9694,6 @@
           <t>Elk Scat</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -9668,7 +9719,6 @@
           <t>Elk Tracks</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -9694,7 +9744,6 @@
           <t>Elk Trail</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -9720,7 +9769,6 @@
           <t>Fox Tracks</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -9776,7 +9824,6 @@
           <t>Squirrel Sighting</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -9802,7 +9849,6 @@
           <t>Wolf Tracks</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -9858,7 +9904,6 @@
           <t>Shed Antler (Deer)</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -9884,7 +9929,6 @@
           <t>Owl/Raptor Feeding Sign on Remains</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -9910,7 +9954,6 @@
           <t>Abandoned / Inactive Bird Nest</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -9936,7 +9979,6 @@
           <t>Moose Browse / Feeding Sign</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -9992,7 +10034,6 @@
           <t>Shed Antler (Moose)</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -10018,7 +10059,6 @@
           <t>Scat / Droppings (Unidentified)</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -10074,7 +10114,6 @@
           <t>Hair / Fur (Unidentified)</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -10160,7 +10199,6 @@
           <t>Grouse Sighting</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -10186,7 +10224,6 @@
           <t>Squirrel Drey (Nest)</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -10212,7 +10249,6 @@
           <t>Squirrel Feeding Sign</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -10238,7 +10274,6 @@
           <t>Ungulate Rub</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -10264,7 +10299,6 @@
           <t>Ungulate Scrape</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -10290,7 +10324,6 @@
           <t>Ungulate Tracks</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -10316,7 +10349,6 @@
           <t>Ungulate Trail</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -10372,7 +10404,6 @@
           <t>Large Game Tracks</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10398,7 +10429,6 @@
           <t>Medium Game Tracks</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10454,7 +10484,6 @@
           <t>Small Game Tracks</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10510,7 +10539,6 @@
           <t>Small Game Trail</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10596,7 +10624,6 @@
           <t>Grouse (Mentioned)</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10652,7 +10679,6 @@
           <t>Game Tracks</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -10678,7 +10704,6 @@
           <t>Game Trail</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -10704,7 +10729,6 @@
           <t>Unidentified Wildlife Tracks</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -10850,7 +10874,6 @@
           <t>Animal Foot Traffic / Active Path</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10999,6 +11022,126 @@
       <c r="F92" t="inlineStr">
         <is>
           <t>Last-resort fallback for any trail/path mention</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>12</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>(?=.*\bsquirrel\b)(?=.*\b(track|tracks|print|prints)\b).*</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Squirrel</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Squirrel Tracks</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Keeps squirrel track observations from falling through to the generic unidentified-track fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>12</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>(?=.*\bbeaver\b)(?=.*\bden(s)?\b).*</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Beaver</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Lodge / Structure</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Beaver Den</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Accept Beaver Den as entered instead of the generic den fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>10</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>(?=.*\b(rabbit|hare)\b)(?=.*\bburrow(s)?\b).*</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Burrow</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare burrow</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Maps hare/rabbit burrow observations to Snowshoe Hare burrow before any generic fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>10</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>(?=.*\b(rabbit|hare)\b)(?=.*\b(feed|feeding)\b).*</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Feeding</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Feeding</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Maps hare/rabbit feeding observations to Snowshoe Hare Feeding.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Hares_Tracks Snowshoe Hare alias
</commit_message>
<xml_diff>
--- a/wls_program/src/WildlifeSweeps/wildlife_parsing_codex_lookup.xlsx
+++ b/wls_program/src/WildlifeSweeps/wildlife_parsing_codex_lookup.xlsx
@@ -1534,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8561,6 +8561,31 @@
       <c r="E281" t="inlineStr">
         <is>
           <t>Snowshoe Hare Feeding</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>10</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>hares tracks</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
     </row>
@@ -8575,7 +8600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11142,6 +11167,36 @@
       <c r="F96" t="inlineStr">
         <is>
           <t>Maps hare/rabbit feeding observations to Snowshoe Hare Feeding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>10</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>(?=.*\bhares\b)(?=.*\b(track|tracks|print|prints)\b).*</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Snowshoe Hare Tracks</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Maps plural hare track entries like 'Hares_Tracks' to the canonical Snowshoe Hare track description.</t>
         </is>
       </c>
     </row>

</xml_diff>